<commit_message>
quelque modification sur le request apprenant tuteur
</commit_message>
<xml_diff>
--- a/resources/Programmes/programmeclasseCE1.xlsx
+++ b/resources/Programmes/programmeclasseCE1.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\JANGAA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\colyl\Documents\Alymia\Gestion scolaire\Back\Gestion-Scolaire\resources\Programmes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70616FAF-9D46-4DBC-B9E0-36BBC72821B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11280"/>
   </bookViews>
   <sheets>
     <sheet name="Feuille 1" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="154">
   <si>
     <t>Matière</t>
   </si>
@@ -500,12 +499,18 @@
   </si>
   <si>
     <t>60 mn</t>
+  </si>
+  <si>
+    <t>Null</t>
+  </si>
+  <si>
+    <t>NULL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d\.m"/>
   </numFmts>
@@ -792,14 +797,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:AA36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="21.33203125" customWidth="1"/>
+    <col min="4" max="4" width="20.88671875" customWidth="1"/>
+    <col min="5" max="5" width="21.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" customWidth="1"/>
+    <col min="8" max="8" width="27.109375" customWidth="1"/>
+    <col min="9" max="9" width="25.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -846,7 +859,7 @@
       <c r="Z1" s="3"/>
       <c r="AA1" s="3"/>
     </row>
-    <row r="2" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -875,7 +888,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:27" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>18</v>
       </c>
@@ -901,7 +914,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:27" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>25</v>
       </c>
@@ -927,7 +940,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:27" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>31</v>
       </c>
@@ -953,7 +966,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>37</v>
       </c>
@@ -979,7 +992,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
         <v>42</v>
       </c>
@@ -1005,7 +1018,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:27" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:27" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>48</v>
       </c>
@@ -1031,7 +1044,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:27" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>54</v>
       </c>
@@ -1060,7 +1073,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:27" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B11" s="5" t="s">
         <v>61</v>
       </c>
@@ -1086,10 +1099,13 @@
         <v>60</v>
       </c>
     </row>
-    <row r="13" spans="1:27" ht="99.75" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:27" ht="55.2" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>66</v>
       </c>
+      <c r="B13" s="5" t="s">
+        <v>152</v>
+      </c>
       <c r="C13" s="5" t="s">
         <v>67</v>
       </c>
@@ -1112,7 +1128,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15" spans="1:27" ht="57" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:27" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>74</v>
       </c>
@@ -1141,7 +1157,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:27" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>81</v>
       </c>
@@ -1159,7 +1175,7 @@
       <c r="H16" s="7"/>
       <c r="I16" s="7"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" ht="41.4" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>85</v>
       </c>
@@ -1188,7 +1204,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="41.4" x14ac:dyDescent="0.25">
       <c r="B19" s="5" t="s">
         <v>93</v>
       </c>
@@ -1214,7 +1230,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B20" s="5" t="s">
         <v>98</v>
       </c>
@@ -1240,7 +1256,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B21" s="5" t="s">
         <v>104</v>
       </c>
@@ -1266,10 +1282,13 @@
         <v>103</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="55.2" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>110</v>
       </c>
+      <c r="B23" s="5" t="s">
+        <v>153</v>
+      </c>
       <c r="C23" s="5" t="s">
         <v>111</v>
       </c>
@@ -1292,10 +1311,13 @@
         <v>116</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="99.75" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" ht="55.2" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>117</v>
       </c>
+      <c r="B25" s="5" t="s">
+        <v>153</v>
+      </c>
       <c r="C25" s="5" t="s">
         <v>118</v>
       </c>
@@ -1318,10 +1340,13 @@
         <v>116</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" ht="55.2" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>122</v>
       </c>
+      <c r="B27" t="s">
+        <v>153</v>
+      </c>
       <c r="C27" s="5" t="s">
         <v>123</v>
       </c>
@@ -1344,7 +1369,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="57" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
         <v>127</v>
       </c>
@@ -1373,7 +1398,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="57" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B31" s="5" t="s">
         <v>132</v>
       </c>
@@ -1391,7 +1416,7 @@
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
     </row>
-    <row r="33" spans="1:9" ht="57" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="27.6" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
         <v>136</v>
       </c>
@@ -1420,7 +1445,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="42.75" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" ht="27.6" x14ac:dyDescent="0.25">
       <c r="B34" s="5" t="s">
         <v>141</v>
       </c>
@@ -1438,9 +1463,12 @@
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
     </row>
-    <row r="36" spans="1:9" ht="128.25" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" ht="55.2" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>145</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>153</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>146</v>

</xml_diff>